<commit_message>
Ajustes resumen por proceso
</commit_message>
<xml_diff>
--- a/data/raw/Subproceso-Proceso-Area.xlsx
+++ b/data/raw/Subproceso-Proceso-Area.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://poligran-my.sharepoint.com/personal/lxisilva_poligran_edu_co/Documents/Documentos/Proyectos/Sistema_Indicadores_Poli/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f15395a9ed9a48f/Proyectos_DS/Sistema_Indicadores_Poli/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="442" documentId="13_ncr:1_{7D5D2E2B-8870-4A5C-A9AF-FD632C2BB311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1123AD19-A07D-48F3-853B-78A107DAFFA3}"/>
@@ -2971,7 +2971,7 @@
     <cfRule type="duplicateValues" dxfId="7" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C54">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -4279,10 +4279,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C55">
-    <cfRule type="duplicateValues" dxfId="5" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="9"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5773,10 +5773,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B56">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C3">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -6558,7 +6558,7 @@
     </filterColumn>
   </autoFilter>
   <conditionalFormatting sqref="B2:B52">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7634,7 +7634,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B53">
-    <cfRule type="duplicateValues" dxfId="1" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="7"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8299,15 +8299,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101004B3553A73F55864994CAF6806DB2233B" ma:contentTypeVersion="15" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="0772d54a1d010170e6fbd4301e22082d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="787dcc16-ad9c-4aed-8595-d8b714944830" xmlns:ns3="eb4e1f33-0654-4877-a695-74ac1243131b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d309db89fd7fb813f1d992ce290f04b6" ns2:_="" ns3:_="">
     <xsd:import namespace="787dcc16-ad9c-4aed-8595-d8b714944830"/>
@@ -8542,6 +8533,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50A7858D-C4BB-4738-AFE6-ACA2D8E7AA74}">
   <ds:schemaRefs>
@@ -8554,14 +8554,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE277362-6D14-47AE-9D5E-D8EAD6BC850B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D12D41D8-D34A-4C1F-82E4-8461693B79B3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -8578,4 +8570,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DE277362-6D14-47AE-9D5E-D8EAD6BC850B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>